<commit_message>
fix(excel): map PS slots past Disposizione and lunch by row offset
Align app slots 1-6 to Desktop 66_PS teaching rows; keep Disposizione and yellow pausa fixed; module text stays black.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/build/web/assets/assets/templates/ps_weekly_blank.xlsx
+++ b/build/web/assets/assets/templates/ps_weekly_blank.xlsx
@@ -13053,7 +13053,7 @@
       <c r="K17" s="560"/>
       <c r="L17" s="546"/>
       <c r="M17" s="541"/>
-      <c r="N17" s="1230"/>
+      <c r="N17" s="1255"/>
       <c r="O17" s="1253"/>
       <c r="P17" s="531"/>
       <c r="AA17" s="531"/>
@@ -13389,7 +13389,7 @@
       <c r="K31" s="576"/>
       <c r="L31" s="576"/>
       <c r="M31" s="576"/>
-      <c r="N31" s="1230"/>
+      <c r="N31" s="1249"/>
       <c r="O31" s="1231"/>
       <c r="Q31" s="531"/>
       <c r="S31" s="531"/>
@@ -13429,7 +13429,7 @@
       <c r="K33" s="560"/>
       <c r="L33" s="546"/>
       <c r="M33" s="541"/>
-      <c r="N33" s="1230"/>
+      <c r="N33" s="1255"/>
       <c r="O33" s="1253"/>
       <c r="P33" s="531"/>
       <c r="Q33" s="531"/>
@@ -13643,7 +13643,7 @@
       <c r="K41" s="560"/>
       <c r="L41" s="546"/>
       <c r="M41" s="541"/>
-      <c r="N41" s="1230"/>
+      <c r="N41" s="1232"/>
       <c r="O41" s="1233"/>
       <c r="P41" s="531"/>
       <c r="Q41" s="531"/>
@@ -13675,7 +13675,7 @@
       <c r="K42" s="560"/>
       <c r="L42" s="546"/>
       <c r="M42" s="541"/>
-      <c r="N42" s="1230"/>
+      <c r="N42" s="1257"/>
       <c r="O42" s="1247"/>
       <c r="R42" s="531"/>
       <c r="S42" s="531"/>
@@ -13705,7 +13705,7 @@
       <c r="K43" s="560"/>
       <c r="L43" s="546"/>
       <c r="M43" s="541"/>
-      <c r="N43" s="1230"/>
+      <c r="N43" s="1249"/>
       <c r="O43" s="1231"/>
       <c r="P43" s="531"/>
       <c r="Q43" s="531"/>
@@ -13738,7 +13738,7 @@
       <c r="K44" s="560"/>
       <c r="L44" s="546"/>
       <c r="M44" s="541"/>
-      <c r="N44" s="1230"/>
+      <c r="N44" s="1252"/>
       <c r="O44" s="1253"/>
       <c r="P44" s="531"/>
       <c r="Q44" s="531"/>

</xml_diff>

<commit_message>
feat(planner): recuperi per bisogno reale, calendario settimane, indicatore assenti
- Dialog recupero: mostra solo frequentatori e moduli con ore da recuperare
  (toRecoverT/P di computePerModuleStats), filtro bidirezionale modulo <->
  frequentatore, scelta teoria/pratica quando servono entrambe, salvataggio
  con recoveredType.
- Header planner: la data settimana apre un calendario per saltare a
  qualsiasi settimana, pulsante "settimana corrente".
- Lezioni con assenti: badge persona-off con conteggio accanto alla
  validazione e cognomi nel tooltip.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/web/assets/assets/templates/ps_weekly_blank.xlsx
+++ b/build/web/assets/assets/templates/ps_weekly_blank.xlsx
@@ -3494,121 +3494,121 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6366F1"/>
+        <fgColor rgb="FFE3E3FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF3B82F6"/>
+        <fgColor rgb="FFDCE8FD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF06B6D4"/>
+        <fgColor rgb="FFD2F2F7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF14B8A6"/>
+        <fgColor rgb="FFD5F2EF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF22C55E"/>
+        <fgColor rgb="FFD7F5E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF84CC16"/>
+        <fgColor rgb="FFE9F6D5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF59E0B"/>
+        <fgColor rgb="FFFDEED3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF97316"/>
+        <fgColor rgb="FFFEE6D5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEF4444"/>
+        <fgColor rgb="FFFCDDDD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEC4899"/>
+        <fgColor rgb="FFFCDEED"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA855F7"/>
+        <fgColor rgb="FFEFE0FE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8B5CF6"/>
+        <fgColor rgb="FFEAE2FD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0EA5E9"/>
+        <fgColor rgb="FFD4EFFB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF10B981"/>
+        <fgColor rgb="FFD4F2E8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD97706"/>
+        <fgColor rgb="FFF8E7D2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF64748B"/>
+        <fgColor rgb="FFE3E6EA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF78716C"/>
+        <fgColor rgb="FFE7E5E5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF854D0E"/>
+        <fgColor rgb="FFE9DFD4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF166534"/>
+        <fgColor rgb="FFD5E3DA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6B7280"/>
+        <fgColor rgb="FFE4E6E8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>

<commit_message>
feat(corsi): admin modifica la data degli aggiornamenti professionali istruttori
Dettaglio istruttore: ogni voce di aggiornamento professionale ha il pulsante
"Modifica data" (date picker); mostrate anche le voci fuori finestra (sbiadite)
per poterne correggere la data. GradeService.updateUpdateDate salva solo la data.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pa86X86fMDND5NTe4KQQGA
</commit_message>
<xml_diff>
--- a/build/web/assets/assets/templates/ps_weekly_blank.xlsx
+++ b/build/web/assets/assets/templates/ps_weekly_blank.xlsx
@@ -2243,10 +2243,10 @@
     <t>C.le Magg. FERDINANDO AVELLO</t>
   </si>
   <si>
-    <t>GRADO, NOME e COGNOME (ESERCITO)</t>
-  </si>
-  <si>
-    <t>GRADO, NOME e COGNOME (CARABINIERI)</t>
+    <t>NOME e COGNOME</t>
+  </si>
+  <si>
+    <t>NOME e COGNOME</t>
   </si>
   <si>
     <t>C.le Magg. OSKAR FONTANA</t>
@@ -13892,7 +13892,7 @@
       <c r="L49" s="1220"/>
       <c r="M49" s="1220"/>
       <c r="N49" s="1220"/>
-      <c r="O49" s="1220"/>
+      <c r="O49" s="1221"/>
       <c r="P49" s="488"/>
     </row>
     <row r="50" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13909,7 +13909,7 @@
       <c r="L50" s="1224"/>
       <c r="M50" s="1224"/>
       <c r="N50" s="1224"/>
-      <c r="O50" s="1224"/>
+      <c r="O50" s="1256"/>
       <c r="P50" s="488"/>
     </row>
     <row r="51" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13942,7 +13942,7 @@
       <c r="L52" s="1216"/>
       <c r="M52" s="1216"/>
       <c r="N52" s="1216"/>
-      <c r="O52" s="1216"/>
+      <c r="O52" s="1217"/>
       <c r="P52" s="488"/>
     </row>
     <row r="53" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13975,7 +13975,7 @@
       <c r="L54" s="1216"/>
       <c r="M54" s="1216"/>
       <c r="N54" s="1216"/>
-      <c r="O54" s="1216"/>
+      <c r="O54" s="1217"/>
       <c r="P54" s="488"/>
     </row>
     <row r="55" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13991,7 +13991,7 @@
       <c r="L55" s="1216"/>
       <c r="M55" s="1216"/>
       <c r="N55" s="1216"/>
-      <c r="O55" s="1216"/>
+      <c r="O55" s="1217"/>
       <c r="P55" s="488"/>
     </row>
     <row r="56" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -14008,7 +14008,7 @@
       <c r="L56" s="1216"/>
       <c r="M56" s="1216"/>
       <c r="N56" s="1216"/>
-      <c r="O56" s="1216"/>
+      <c r="O56" s="1217"/>
       <c r="P56" s="488"/>
     </row>
     <row r="57" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -14025,7 +14025,7 @@
       <c r="L57" s="1216"/>
       <c r="M57" s="1216"/>
       <c r="N57" s="1216"/>
-      <c r="O57" s="1216"/>
+      <c r="O57" s="1217"/>
       <c r="P57" s="488"/>
     </row>
     <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>